<commit_message>
ETL Testing complete till "Programs"
</commit_message>
<xml_diff>
--- a/resources/locations.xlsx
+++ b/resources/locations.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\ETB_TAJIKISTAN_OPENMRS\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owais\workspace\openmrs-mdrtb-etl-job\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A99529-80B2-47CE-A86A-7AE917AFDF29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E625817-E825-4E1D-8BD3-6D58703C6D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6F8C5509-F00C-4DDA-A378-947946C44FBF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6F8C5509-F00C-4DDA-A378-947946C44FBF}"/>
   </bookViews>
   <sheets>
-    <sheet name="Locations" sheetId="2" r:id="rId1"/>
+    <sheet name="locations" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Locations!$A$1:$M$281</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">locations!$A$1:$M$281</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -2332,9 +2332,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2372,7 +2372,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2478,7 +2478,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2620,7 +2620,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2629,24 +2629,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53BFBD4D-E460-4B5B-B884-F960F6E32D71}">
   <dimension ref="A1:M283"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="53.5546875" customWidth="1"/>
-    <col min="3" max="3" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="43.33203125" customWidth="1"/>
-    <col min="6" max="6" width="18.21875" customWidth="1"/>
-    <col min="7" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.21875" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="39.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="53.5703125" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43.28515625" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="39.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>1</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -2712,7 +2712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -2743,7 +2743,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -2774,7 +2774,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
         <v>4</v>
       </c>
@@ -2805,7 +2805,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -2832,7 +2832,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="7" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
         <v>6</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
         <v>7</v>
       </c>
@@ -2894,7 +2894,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
         <v>8</v>
       </c>
@@ -2925,7 +2925,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
         <v>9</v>
       </c>
@@ -2956,7 +2956,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -2987,7 +2987,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -3018,7 +3018,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -3049,7 +3049,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -3111,7 +3111,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -3142,7 +3142,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -3173,7 +3173,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>17</v>
       </c>
@@ -3206,7 +3206,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>18</v>
       </c>
@@ -3237,7 +3237,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>19</v>
       </c>
@@ -3268,7 +3268,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <v>20</v>
       </c>
@@ -3299,7 +3299,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>21</v>
       </c>
@@ -3330,7 +3330,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>22</v>
       </c>
@@ -3361,7 +3361,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9">
         <v>23</v>
       </c>
@@ -3396,7 +3396,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9">
         <v>24</v>
       </c>
@@ -3431,7 +3431,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>25</v>
       </c>
@@ -3462,7 +3462,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="27" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="9">
         <v>26</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="28" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9">
         <v>27</v>
       </c>
@@ -3532,7 +3532,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <v>28</v>
       </c>
@@ -3563,7 +3563,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -3594,7 +3594,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <v>30</v>
       </c>
@@ -3625,7 +3625,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <v>31</v>
       </c>
@@ -3656,7 +3656,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
         <v>32</v>
       </c>
@@ -3687,7 +3687,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
         <v>33</v>
       </c>
@@ -3718,7 +3718,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="4">
         <v>34</v>
       </c>
@@ -3749,7 +3749,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
         <v>35</v>
       </c>
@@ -3780,7 +3780,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="4">
         <v>36</v>
       </c>
@@ -3811,7 +3811,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="4">
         <v>37</v>
       </c>
@@ -3842,7 +3842,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="4">
         <v>38</v>
       </c>
@@ -3873,7 +3873,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="4">
         <v>39</v>
       </c>
@@ -3904,7 +3904,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="4">
         <v>40</v>
       </c>
@@ -3935,7 +3935,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="4">
         <v>41</v>
       </c>
@@ -3966,7 +3966,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="4">
         <v>42</v>
       </c>
@@ -3997,7 +3997,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="44" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="9">
         <v>43</v>
       </c>
@@ -4032,7 +4032,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="4">
         <v>44</v>
       </c>
@@ -4063,7 +4063,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="4">
         <v>45</v>
       </c>
@@ -4094,7 +4094,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" s="4">
         <v>46</v>
       </c>
@@ -4125,7 +4125,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="4">
         <v>47</v>
       </c>
@@ -4156,7 +4156,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" s="4">
         <v>48</v>
       </c>
@@ -4187,7 +4187,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" s="4">
         <v>49</v>
       </c>
@@ -4218,7 +4218,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" s="4">
         <v>50</v>
       </c>
@@ -4249,7 +4249,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" s="4">
         <v>51</v>
       </c>
@@ -4280,7 +4280,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" s="4">
         <v>52</v>
       </c>
@@ -4311,7 +4311,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" s="4">
         <v>53</v>
       </c>
@@ -4342,7 +4342,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" s="4">
         <v>54</v>
       </c>
@@ -4373,7 +4373,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" s="4">
         <v>55</v>
       </c>
@@ -4404,7 +4404,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" s="4">
         <v>56</v>
       </c>
@@ -4435,7 +4435,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" s="4">
         <v>57</v>
       </c>
@@ -4466,7 +4466,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" s="4">
         <v>58</v>
       </c>
@@ -4497,7 +4497,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" s="4">
         <v>59</v>
       </c>
@@ -4528,7 +4528,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" s="4">
         <v>60</v>
       </c>
@@ -4559,7 +4559,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="62" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="9">
         <v>61</v>
       </c>
@@ -4594,7 +4594,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A63" s="4">
         <v>62</v>
       </c>
@@ -4625,7 +4625,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" s="4">
         <v>63</v>
       </c>
@@ -4656,7 +4656,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" s="4">
         <v>64</v>
       </c>
@@ -4687,7 +4687,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" s="4">
         <v>65</v>
       </c>
@@ -4718,7 +4718,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" s="4">
         <v>66</v>
       </c>
@@ -4749,7 +4749,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
         <v>67</v>
       </c>
@@ -4780,7 +4780,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A69" s="4">
         <v>68</v>
       </c>
@@ -4811,7 +4811,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="70" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="9">
         <v>69</v>
       </c>
@@ -4846,7 +4846,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="71" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="9">
         <v>70</v>
       </c>
@@ -4881,7 +4881,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="72" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="9">
         <v>71</v>
       </c>
@@ -4916,7 +4916,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" s="4">
         <v>72</v>
       </c>
@@ -4947,7 +4947,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" s="4">
         <v>73</v>
       </c>
@@ -4978,7 +4978,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" s="4">
         <v>74</v>
       </c>
@@ -5009,7 +5009,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" s="4">
         <v>75</v>
       </c>
@@ -5040,7 +5040,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" s="4">
         <v>76</v>
       </c>
@@ -5071,7 +5071,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" s="4">
         <v>77</v>
       </c>
@@ -5102,7 +5102,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" s="4">
         <v>78</v>
       </c>
@@ -5133,7 +5133,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
         <v>79</v>
       </c>
@@ -5164,7 +5164,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A81" s="4">
         <v>80</v>
       </c>
@@ -5195,7 +5195,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
         <v>81</v>
       </c>
@@ -5226,7 +5226,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A83" s="4">
         <v>82</v>
       </c>
@@ -5257,7 +5257,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
         <v>83</v>
       </c>
@@ -5288,7 +5288,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A85" s="4">
         <v>84</v>
       </c>
@@ -5319,7 +5319,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A86" s="4">
         <v>85</v>
       </c>
@@ -5350,7 +5350,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="87" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="9">
         <v>86</v>
       </c>
@@ -5383,7 +5383,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="88" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="9">
         <v>87</v>
       </c>
@@ -5414,7 +5414,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="89" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="9">
         <v>88</v>
       </c>
@@ -5451,7 +5451,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="90" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="9">
         <v>89</v>
       </c>
@@ -5486,7 +5486,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="91" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="9">
         <v>90</v>
       </c>
@@ -5521,7 +5521,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="92" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="9">
         <v>91</v>
       </c>
@@ -5556,7 +5556,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="93" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="9">
         <v>92</v>
       </c>
@@ -5591,7 +5591,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="94" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="9">
         <v>93</v>
       </c>
@@ -5622,7 +5622,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="95" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="9">
         <v>94</v>
       </c>
@@ -5655,7 +5655,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="96" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="9">
         <v>95</v>
       </c>
@@ -5690,7 +5690,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A97" s="4">
         <v>96</v>
       </c>
@@ -5721,7 +5721,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A98" s="4">
         <v>97</v>
       </c>
@@ -5752,7 +5752,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A99" s="4">
         <v>98</v>
       </c>
@@ -5783,7 +5783,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
         <v>99</v>
       </c>
@@ -5814,7 +5814,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
         <v>100</v>
       </c>
@@ -5845,7 +5845,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
         <v>101</v>
       </c>
@@ -5876,7 +5876,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
         <v>102</v>
       </c>
@@ -5907,7 +5907,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
         <v>103</v>
       </c>
@@ -5938,7 +5938,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
         <v>104</v>
       </c>
@@ -5969,7 +5969,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="106" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="9">
         <v>105</v>
       </c>
@@ -6004,7 +6004,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
         <v>106</v>
       </c>
@@ -6035,7 +6035,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
         <v>107</v>
       </c>
@@ -6066,7 +6066,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
         <v>108</v>
       </c>
@@ -6097,7 +6097,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
         <v>109</v>
       </c>
@@ -6128,7 +6128,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
         <v>110</v>
       </c>
@@ -6159,7 +6159,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
         <v>111</v>
       </c>
@@ -6190,7 +6190,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="113" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="9">
         <v>112</v>
       </c>
@@ -6225,7 +6225,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="114" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="9">
         <v>113</v>
       </c>
@@ -6260,7 +6260,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="115" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="9">
         <v>114</v>
       </c>
@@ -6295,7 +6295,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="116" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="9">
         <v>115</v>
       </c>
@@ -6326,7 +6326,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="117" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="9">
         <v>116</v>
       </c>
@@ -6363,7 +6363,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="118" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="9">
         <v>117</v>
       </c>
@@ -6400,7 +6400,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="119" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="9">
         <v>118</v>
       </c>
@@ -6437,7 +6437,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="120" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="9">
         <v>119</v>
       </c>
@@ -6474,7 +6474,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="121" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="9">
         <v>120</v>
       </c>
@@ -6511,7 +6511,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="122" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="9">
         <v>121</v>
       </c>
@@ -6548,7 +6548,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="123" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="9">
         <v>122</v>
       </c>
@@ -6585,7 +6585,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="124" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="9">
         <v>123</v>
       </c>
@@ -6620,7 +6620,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="125" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="9">
         <v>124</v>
       </c>
@@ -6655,7 +6655,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="126" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="9">
         <v>125</v>
       </c>
@@ -6692,7 +6692,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="127" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="9">
         <v>126</v>
       </c>
@@ -6723,7 +6723,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="128" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="9">
         <v>127</v>
       </c>
@@ -6754,7 +6754,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="129" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="9">
         <v>128</v>
       </c>
@@ -6789,7 +6789,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="130" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="9">
         <v>129</v>
       </c>
@@ -6826,7 +6826,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="131" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="9">
         <v>130</v>
       </c>
@@ -6863,7 +6863,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="132" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="9">
         <v>131</v>
       </c>
@@ -6900,7 +6900,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="133" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="9">
         <v>132</v>
       </c>
@@ -6931,7 +6931,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="134" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="9">
         <v>133</v>
       </c>
@@ -6966,7 +6966,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="135" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="9">
         <v>134</v>
       </c>
@@ -7003,7 +7003,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="136" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="9">
         <v>135</v>
       </c>
@@ -7034,7 +7034,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="137" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="9">
         <v>136</v>
       </c>
@@ -7071,7 +7071,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="138" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="9">
         <v>137</v>
       </c>
@@ -7108,7 +7108,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="139" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="9">
         <v>138</v>
       </c>
@@ -7145,7 +7145,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="140" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="9">
         <v>139</v>
       </c>
@@ -7182,7 +7182,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="141" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="9">
         <v>140</v>
       </c>
@@ -7219,7 +7219,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="142" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="9">
         <v>141</v>
       </c>
@@ -7256,7 +7256,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="143" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="9">
         <v>142</v>
       </c>
@@ -7293,7 +7293,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="144" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="9">
         <v>143</v>
       </c>
@@ -7330,7 +7330,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="145" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="9">
         <v>144</v>
       </c>
@@ -7365,7 +7365,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="146" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="9">
         <v>145</v>
       </c>
@@ -7400,7 +7400,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="147" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="9">
         <v>146</v>
       </c>
@@ -7431,7 +7431,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="148" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A148" s="9">
         <v>147</v>
       </c>
@@ -7468,7 +7468,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="149" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="9">
         <v>148</v>
       </c>
@@ -7505,7 +7505,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="150" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="9">
         <v>149</v>
       </c>
@@ -7542,7 +7542,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="151" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="9">
         <v>150</v>
       </c>
@@ -7579,7 +7579,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="152" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A152" s="9">
         <v>151</v>
       </c>
@@ -7616,7 +7616,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="153" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A153" s="9">
         <v>152</v>
       </c>
@@ -7647,7 +7647,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="154" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="9">
         <v>153</v>
       </c>
@@ -7684,7 +7684,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="155" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="9">
         <v>154</v>
       </c>
@@ -7721,7 +7721,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="156" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="9">
         <v>155</v>
       </c>
@@ -7758,7 +7758,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="157" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="9">
         <v>156</v>
       </c>
@@ -7795,7 +7795,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="158" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="9">
         <v>157</v>
       </c>
@@ -7826,7 +7826,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="159" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="9">
         <v>158</v>
       </c>
@@ -7863,7 +7863,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="160" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="9">
         <v>159</v>
       </c>
@@ -7894,7 +7894,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="161" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A161" s="9">
         <v>160</v>
       </c>
@@ -7931,7 +7931,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="162" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="9">
         <v>161</v>
       </c>
@@ -7968,7 +7968,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="163" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="9">
         <v>162</v>
       </c>
@@ -8005,7 +8005,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="164" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="9">
         <v>163</v>
       </c>
@@ -8042,7 +8042,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="165" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A165" s="9">
         <v>164</v>
       </c>
@@ -8079,7 +8079,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="166" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="9">
         <v>165</v>
       </c>
@@ -8116,7 +8116,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="167" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="9">
         <v>166</v>
       </c>
@@ -8153,7 +8153,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="168" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="9">
         <v>167</v>
       </c>
@@ -8190,7 +8190,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="169" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="9">
         <v>168</v>
       </c>
@@ -8227,7 +8227,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="170" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A170" s="9">
         <v>169</v>
       </c>
@@ -8264,7 +8264,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="171" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A171" s="9">
         <v>170</v>
       </c>
@@ -8295,7 +8295,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="172" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="9">
         <v>171</v>
       </c>
@@ -8330,7 +8330,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="173" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A173" s="9">
         <v>172</v>
       </c>
@@ -8361,7 +8361,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="174" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A174" s="9">
         <v>173</v>
       </c>
@@ -8392,7 +8392,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="175" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="9">
         <v>174</v>
       </c>
@@ -8429,7 +8429,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="176" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="9">
         <v>175</v>
       </c>
@@ -8466,7 +8466,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="177" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="9">
         <v>176</v>
       </c>
@@ -8503,7 +8503,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="178" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="9">
         <v>177</v>
       </c>
@@ -8540,7 +8540,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="179" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A179" s="9">
         <v>178</v>
       </c>
@@ -8577,7 +8577,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="180" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="9">
         <v>179</v>
       </c>
@@ -8614,7 +8614,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="181" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A181" s="9">
         <v>180</v>
       </c>
@@ -8651,7 +8651,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="182" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A182" s="9">
         <v>181</v>
       </c>
@@ -8688,7 +8688,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="183" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A183" s="9">
         <v>182</v>
       </c>
@@ -8725,7 +8725,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="184" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A184" s="9">
         <v>183</v>
       </c>
@@ -8762,7 +8762,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="185" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A185" s="9">
         <v>184</v>
       </c>
@@ -8799,7 +8799,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="186" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A186" s="9">
         <v>185</v>
       </c>
@@ -8836,7 +8836,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="187" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A187" s="4">
         <v>186</v>
       </c>
@@ -8867,7 +8867,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="188" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A188" s="4">
         <v>187</v>
       </c>
@@ -8898,7 +8898,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="189" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A189" s="4">
         <v>188</v>
       </c>
@@ -8929,7 +8929,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="190" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A190" s="4">
         <v>189</v>
       </c>
@@ -8960,7 +8960,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="191" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A191" s="4">
         <v>190</v>
       </c>
@@ -8991,7 +8991,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="192" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A192" s="4">
         <v>191</v>
       </c>
@@ -9022,7 +9022,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="193" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A193" s="4">
         <v>192</v>
       </c>
@@ -9053,7 +9053,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="194" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="9">
         <v>193</v>
       </c>
@@ -9088,7 +9088,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="195" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="9">
         <v>194</v>
       </c>
@@ -9123,7 +9123,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="196" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="9">
         <v>195</v>
       </c>
@@ -9158,7 +9158,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="197" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="9">
         <v>196</v>
       </c>
@@ -9193,7 +9193,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="198" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="9">
         <v>197</v>
       </c>
@@ -9228,7 +9228,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="199" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="9">
         <v>198</v>
       </c>
@@ -9263,7 +9263,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="200" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A200" s="4">
         <v>199</v>
       </c>
@@ -9294,7 +9294,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="201" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A201" s="4">
         <v>200</v>
       </c>
@@ -9325,7 +9325,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="202" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A202" s="4">
         <v>201</v>
       </c>
@@ -9356,7 +9356,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="203" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A203" s="4">
         <v>202</v>
       </c>
@@ -9387,7 +9387,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="204" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A204" s="4">
         <v>203</v>
       </c>
@@ -9418,7 +9418,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="205" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A205" s="4">
         <v>204</v>
       </c>
@@ -9449,7 +9449,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="206" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A206" s="9">
         <v>205</v>
       </c>
@@ -9484,7 +9484,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="207" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A207" s="4">
         <v>206</v>
       </c>
@@ -9513,7 +9513,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="208" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A208" s="4">
         <v>207</v>
       </c>
@@ -9542,7 +9542,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="209" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A209" s="4">
         <v>208</v>
       </c>
@@ -9571,7 +9571,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="210" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A210" s="4">
         <v>209</v>
       </c>
@@ -9600,7 +9600,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="211" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A211" s="4">
         <v>210</v>
       </c>
@@ -9629,7 +9629,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="212" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A212" s="4">
         <v>211</v>
       </c>
@@ -9658,7 +9658,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="213" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A213" s="4">
         <v>212</v>
       </c>
@@ -9687,7 +9687,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="214" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A214" s="4">
         <v>213</v>
       </c>
@@ -9716,7 +9716,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="215" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A215" s="4">
         <v>214</v>
       </c>
@@ -9745,7 +9745,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="216" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A216" s="9">
         <v>215</v>
       </c>
@@ -9780,7 +9780,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="217" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A217" s="9">
         <v>216</v>
       </c>
@@ -9815,7 +9815,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="218" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A218" s="9">
         <v>217</v>
       </c>
@@ -9850,7 +9850,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="219" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A219" s="9">
         <v>218</v>
       </c>
@@ -9885,7 +9885,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="220" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A220" s="9">
         <v>219</v>
       </c>
@@ -9920,7 +9920,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="221" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A221" s="9">
         <v>220</v>
       </c>
@@ -9955,7 +9955,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="222" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A222" s="9">
         <v>221</v>
       </c>
@@ -9990,7 +9990,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="223" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A223" s="9">
         <v>222</v>
       </c>
@@ -10025,7 +10025,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="224" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A224" s="4">
         <v>223</v>
       </c>
@@ -10054,7 +10054,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="225" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A225" s="4">
         <v>224</v>
       </c>
@@ -10083,7 +10083,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="226" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A226" s="9">
         <v>225</v>
       </c>
@@ -10118,7 +10118,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="227" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A227" s="9">
         <v>226</v>
       </c>
@@ -10153,7 +10153,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="228" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A228" s="9">
         <v>227</v>
       </c>
@@ -10188,7 +10188,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="229" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A229" s="9">
         <v>228</v>
       </c>
@@ -10223,7 +10223,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="230" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A230" s="9">
         <v>229</v>
       </c>
@@ -10258,7 +10258,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="231" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A231" s="9">
         <v>230</v>
       </c>
@@ -10293,7 +10293,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="232" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A232" s="9">
         <v>231</v>
       </c>
@@ -10328,7 +10328,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="233" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A233" s="9">
         <v>232</v>
       </c>
@@ -10363,7 +10363,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="234" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A234" s="9">
         <v>233</v>
       </c>
@@ -10398,7 +10398,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="235" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A235" s="9">
         <v>234</v>
       </c>
@@ -10433,7 +10433,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="236" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A236" s="9">
         <v>235</v>
       </c>
@@ -10468,7 +10468,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="237" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A237" s="9">
         <v>236</v>
       </c>
@@ -10503,7 +10503,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="238" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A238" s="9">
         <v>237</v>
       </c>
@@ -10538,7 +10538,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="239" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A239" s="9">
         <v>238</v>
       </c>
@@ -10573,7 +10573,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="240" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A240" s="9">
         <v>239</v>
       </c>
@@ -10608,7 +10608,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="241" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A241" s="9">
         <v>240</v>
       </c>
@@ -10643,7 +10643,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="242" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A242" s="9">
         <v>241</v>
       </c>
@@ -10678,7 +10678,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="243" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A243" s="9">
         <v>242</v>
       </c>
@@ -10713,7 +10713,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="244" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A244" s="9">
         <v>243</v>
       </c>
@@ -10748,7 +10748,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="245" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A245" s="9">
         <v>244</v>
       </c>
@@ -10783,7 +10783,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="246" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A246" s="9">
         <v>245</v>
       </c>
@@ -10818,7 +10818,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="247" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A247" s="9">
         <v>246</v>
       </c>
@@ -10853,7 +10853,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="248" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A248" s="9">
         <v>247</v>
       </c>
@@ -10888,7 +10888,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="249" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A249" s="9">
         <v>248</v>
       </c>
@@ -10923,7 +10923,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="250" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A250" s="9">
         <v>249</v>
       </c>
@@ -10958,7 +10958,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="251" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A251" s="9">
         <v>250</v>
       </c>
@@ -10993,7 +10993,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="252" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A252" s="9">
         <v>251</v>
       </c>
@@ -11028,7 +11028,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="253" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A253" s="9">
         <v>252</v>
       </c>
@@ -11063,7 +11063,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="254" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A254" s="9">
         <v>253</v>
       </c>
@@ -11098,7 +11098,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="255" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A255" s="9">
         <v>254</v>
       </c>
@@ -11133,7 +11133,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="256" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A256" s="9">
         <v>255</v>
       </c>
@@ -11168,7 +11168,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="257" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A257" s="9">
         <v>256</v>
       </c>
@@ -11203,7 +11203,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="258" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A258" s="9">
         <v>257</v>
       </c>
@@ -11238,7 +11238,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="259" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A259" s="9">
         <v>258</v>
       </c>
@@ -11273,7 +11273,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="260" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A260" s="9">
         <v>259</v>
       </c>
@@ -11308,7 +11308,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="261" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A261" s="9">
         <v>260</v>
       </c>
@@ -11343,7 +11343,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="262" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A262" s="9">
         <v>261</v>
       </c>
@@ -11378,7 +11378,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="263" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A263" s="9">
         <v>262</v>
       </c>
@@ -11413,7 +11413,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="264" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A264" s="4">
         <v>263</v>
       </c>
@@ -11442,7 +11442,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="265" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A265" s="4">
         <v>264</v>
       </c>
@@ -11471,7 +11471,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="266" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A266" s="4">
         <v>265</v>
       </c>
@@ -11502,7 +11502,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="267" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A267" s="4">
         <v>266</v>
       </c>
@@ -11533,7 +11533,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="268" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A268" s="4">
         <v>267</v>
       </c>
@@ -11564,7 +11564,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="269" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A269" s="4">
         <v>268</v>
       </c>
@@ -11595,7 +11595,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="270" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A270" s="4">
         <v>269</v>
       </c>
@@ -11626,7 +11626,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="271" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A271" s="4">
         <v>270</v>
       </c>
@@ -11657,7 +11657,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="272" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A272" s="4">
         <v>271</v>
       </c>
@@ -11688,7 +11688,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="273" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A273" s="4">
         <v>272</v>
       </c>
@@ -11717,7 +11717,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="274" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A274" s="4">
         <v>273</v>
       </c>
@@ -11746,7 +11746,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="275" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A275" s="4">
         <v>274</v>
       </c>
@@ -11775,7 +11775,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="276" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A276" s="4">
         <v>275</v>
       </c>
@@ -11804,7 +11804,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="277" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A277" s="4">
         <v>276</v>
       </c>
@@ -11833,7 +11833,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="278" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A278" s="4">
         <v>277</v>
       </c>
@@ -11864,7 +11864,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="279" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A279" s="4">
         <v>278</v>
       </c>
@@ -11895,7 +11895,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="280" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A280" s="4">
         <v>279</v>
       </c>
@@ -11926,7 +11926,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="281" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A281" s="4">
         <v>280</v>
       </c>
@@ -11957,7 +11957,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="282" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A282" s="4">
         <v>281</v>
       </c>
@@ -11983,7 +11983,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="283" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A283" s="4">
         <v>282</v>
       </c>

</xml_diff>